<commit_message>
docs(c6.3): align G13 gate status with final PR head
</commit_message>
<xml_diff>
--- a/docs/c6/MealUp_C6.3_Integration_Master_Plan_v17_G13_PR1_COMPLETE.xlsx
+++ b/docs/c6/MealUp_C6.3_Integration_Master_Plan_v17_G13_PR1_COMPLETE.xlsx
@@ -2,37 +2,37 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R06461e858eb04fc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Master" sheetId="2" r:id="R7b82c7fc161f4350"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generation_Backlog" sheetId="3" r:id="Rda8f207efe3b40b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pre_Generation_Gate" sheetId="4" r:id="Rbf8043919ec14746"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Waves" sheetId="5" r:id="Rb857926c996e4b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB01_Post_QA" sheetId="6" r:id="Rd622d47421954640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB02_Post_QA" sheetId="7" r:id="R7be22fb6b9fc4d50"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB03_Post_QA" sheetId="8" r:id="R261bc4b432ba4280"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generation_Log" sheetId="9" r:id="Rff65e14b39444042"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules_Current" sheetId="10" r:id="R39c89b8b226c4c8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing_FO_Plan" sheetId="11" r:id="Re8ac4f11b97741a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB05_Post_QA" sheetId="12" r:id="R48a28c06065043c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB06_Post_QA" sheetId="13" r:id="Rc8cfc194b08049b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closure_Status" sheetId="14" r:id="Rf790f96124bd4c0b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LAMB_Reuse_Test" sheetId="15" r:id="R508c715f36ba4ee3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction_QA_Final" sheetId="16" r:id="R9fed473bdbd8411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping_Final" sheetId="17" r:id="Racbbf5a868cf46db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registration_Final" sheetId="18" r:id="R0ceac95f9aae46f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration_Master_Plan" sheetId="19" r:id="Re04f4e56183b4d27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FO_Surface_Rules" sheetId="20" r:id="R197f8f1f5c934752"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gauge_Contract" sheetId="21" r:id="R19c6c6b369444b53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry_Contract" sheetId="22" r:id="R5560bdfb0be148cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hard_Stops" sheetId="23" r:id="R03f9767401f44112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G0_Freeze_Manifest" sheetId="24" r:id="R7e0932cba2564000"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G1_Recipe_Parity_Audit" sheetId="25" r:id="R15409642f6d24ce1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G2_Registration" sheetId="26" r:id="Rdff310f0a57d4a75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G3_Master_Resolver" sheetId="27" r:id="Rcef1e20e15bb4aa7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G4_Asset_Metrics" sheetId="28" r:id="R1392e49b78834be0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G4_Mapping_Render" sheetId="29" r:id="R2a06a5fa94c9419a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G5_Template_Inventory" sheetId="30" r:id="R2692823b9f454575"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G11_G12_QA" sheetId="31" r:id="R63da8405fa614ecf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rdd31825e15144bf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Audit_Master" sheetId="2" r:id="Rf19b154b34f04690"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generation_Backlog" sheetId="3" r:id="R9635d95a8be94f36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pre_Generation_Gate" sheetId="4" r:id="R0ed4571ac4724416"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production_Waves" sheetId="5" r:id="Rbf0170ba80244023"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB01_Post_QA" sheetId="6" r:id="Rfaa2fdda944043cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB02_Post_QA" sheetId="7" r:id="Rd27aec9668b64bb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB03_Post_QA" sheetId="8" r:id="Rdc5d7e6654da4cc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generation_Log" sheetId="9" r:id="Rc0be123bf6fc4255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rules_Current" sheetId="10" r:id="R9d83000c903e47d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Missing_FO_Plan" sheetId="11" r:id="Rad9dab731f14427f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB05_Post_QA" sheetId="12" r:id="R5f65ae16da6441bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PB06_Post_QA" sheetId="13" r:id="R635f1f2b3c004347"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Closure_Status" sheetId="14" r:id="Re0e359673a3c48c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LAMB_Reuse_Test" sheetId="15" r:id="Rfe1bf5def3534511"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extraction_QA_Final" sheetId="16" r:id="R15db6affd6cf4044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mapping_Final" sheetId="17" r:id="Rd04124a215e64f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Registration_Final" sheetId="18" r:id="Re5c7d89a136b4cb3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Integration_Master_Plan" sheetId="19" r:id="R4bea2f6b99ba4446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FO_Surface_Rules" sheetId="20" r:id="R977b0830ee564ac7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gauge_Contract" sheetId="21" r:id="Rc91f02a349e44907"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Geometry_Contract" sheetId="22" r:id="R49d25501e3dd4080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hard_Stops" sheetId="23" r:id="R43ba988e4f0444d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G0_Freeze_Manifest" sheetId="24" r:id="R1b8e95131f3e4b88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G1_Recipe_Parity_Audit" sheetId="25" r:id="R56407ca490bf4ffd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G2_Registration" sheetId="26" r:id="R1d9ea43e51b045ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G3_Master_Resolver" sheetId="27" r:id="Re1e757cdcbef47a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G4_Asset_Metrics" sheetId="28" r:id="Rb6604b165fcf4d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G4_Mapping_Render" sheetId="29" r:id="Reb0887e8ebeb4b3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G5_Template_Inventory" sheetId="30" r:id="Rbca3ed5443804714"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="G11_G12_QA" sheetId="31" r:id="Rac3c4505c5be463d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1418,7 +1418,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R7a9c0ee01aff4400"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra51adca0e85c423e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1802,7 +1802,7 @@
     <x:mergeCell ref="A12:E12"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61c834ca4de54f85"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50dcbdece4f14539"/>
 </x:worksheet>
 </file>
 
@@ -11674,7 +11674,7 @@
         <x:v>Report finale + screenshot + hash + test</x:v>
       </x:c>
       <x:c r="D17" s="21" t="str">
-        <x:v>G13 approvato il 30/09/2026. Runtime e asset del candidato applicati al branch codex/mealup-c63-g11-g12-g13; commit finale b1f8cb2. PR #1 aperta e mergeable; 2 commit ahead, 0 behind main. Nessun merge o deploy.</x:v>
+        <x:v>G13 approvato il 30/09/2026. Runtime e asset applicati sul branch (commit b1f8cb2); questo masterplan è incluso nella PR #1 aperta e mergeable. 4 commit ahead, 0 behind main. Nessun merge o deploy.</x:v>
       </x:c>
       <x:c r="E17" s="21" t="str">
         <x:v>Regressione rilevata in review o richiesta di modifica.</x:v>
@@ -27487,7 +27487,7 @@
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
       <x:c r="A18" s="324" t="str">
-        <x:v>Branch codex/mealup-c63-g11-g12-g13 aggiornato a b1f8cb2; PR #1 aperta; main non modificato e nessun deploy.</x:v>
+        <x:v>G13 sul branch codex/mealup-c63-g11-g12-g13; masterplan incluso nella PR #1. main non modificato e nessun deploy.</x:v>
       </x:c>
       <x:c r="B18" s="324"/>
       <x:c r="C18" s="324"/>
@@ -27499,10 +27499,10 @@
         <x:v>G13</x:v>
       </x:c>
       <x:c r="B19" s="21" t="str">
-        <x:v>PR #1 — 289 file cambiati, 3 commit ahead / 0 behind</x:v>
+        <x:v>PR #1 — 289 file cambiati, 4 commit ahead / 0 behind</x:v>
       </x:c>
       <x:c r="C19" s="21" t="n">
-        <x:v>3</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D19" s="21" t="str">
         <x:v>OPEN</x:v>

</xml_diff>